<commit_message>
docs: refresh README, onboarding, and test plan/tracker/PDF for v1.8.0 (per-user auth debug + companion dashboards)
</commit_message>
<xml_diff>
--- a/TEST_RESULTS_TRACKER.xlsx
+++ b/TEST_RESULTS_TRACKER.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Test Results" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Results'!$A$1:$H$71</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Results'!$A$1:$H$80</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="269">
   <si>
     <t xml:space="preserve">HPE Networking Assistant — Test Results Summary</t>
   </si>
@@ -32,7 +32,7 @@
     <t xml:space="preserve">Product version</t>
   </si>
   <si>
-    <t xml:space="preserve">1.7.0</t>
+    <t xml:space="preserve">1.8.0</t>
   </si>
   <si>
     <t xml:space="preserve">Tester</t>
@@ -143,7 +143,7 @@
     <t xml:space="preserve">Run pytest -q</t>
   </si>
   <si>
-    <t xml:space="preserve">65 passed</t>
+    <t xml:space="preserve">66 passed</t>
   </si>
   <si>
     <t xml:space="preserve">A3</t>
@@ -488,6 +488,15 @@
     <t xml:space="preserve">Events scoped to that MAC</t>
   </si>
   <si>
+    <t xml:space="preserve">AA-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auth focus by user (username/cert CN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Events scoped to that identity (free-text); failures highlighted</t>
+  </si>
+  <si>
     <t xml:space="preserve">NAC-1</t>
   </si>
   <si>
@@ -527,6 +536,81 @@
     <t xml:space="preserve">Zeros/'No data', no error</t>
   </si>
   <si>
+    <t xml:space="preserve">CD-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Companion dashboards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open Network/NAC dashboard artifact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Device doughnut + cards load from live data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto-refresh ~30s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Updates on its own; last-updated advances; live dot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NAC empty-state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shows 'not configured' rather than erroring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open NAC Auth Debugger artifact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loads with input + time-window controls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debug by username</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pulls identity's NAC events; pass/fail counts; timeline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debug by MAC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto-routes to MAC filter; events returned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD-7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Failure decode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Most-recent-failure card: reason, rule, auth type, NAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explain hand-off</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sends failure detail to chat as a prompt</t>
+  </si>
+  <si>
     <t xml:space="preserve">WR-1</t>
   </si>
   <si>
@@ -746,7 +830,7 @@
     <t xml:space="preserve">SC-5</t>
   </si>
   <si>
-    <t xml:space="preserve">Automated suite 65 passed</t>
+    <t xml:space="preserve">Automated suite 66 passed</t>
   </si>
 </sst>
 </file>
@@ -1214,13 +1298,11 @@
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
@@ -1235,8 +1317,8 @@
         <v>7</v>
       </c>
       <c r="B9" s="3" t="n">
-        <f aca="false">COUNTA('Test Results'!A2:A71)</f>
-        <v>70</v>
+        <f aca="false">COUNTA('Test Results'!A2:A80)</f>
+        <v>79</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1244,7 +1326,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E71,"Pass")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E80,"Pass")</f>
         <v>0</v>
       </c>
     </row>
@@ -1253,7 +1335,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E71,"Fail")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E80,"Fail")</f>
         <v>0</v>
       </c>
     </row>
@@ -1262,7 +1344,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E71,"Blocked")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E80,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
@@ -1271,7 +1353,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E71,"N/A")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E80,"N/A")</f>
         <v>0</v>
       </c>
     </row>
@@ -1281,7 +1363,7 @@
       </c>
       <c r="B14" s="3" t="n">
         <f aca="false">B9-(B10+B11+B12+B13)</f>
-        <v>70</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1309,11 +1391,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
@@ -2103,18 +2185,18 @@
       <c r="G43" s="7"/>
       <c r="H43" s="8"/>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
         <v>154</v>
       </c>
       <c r="B44" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="C44" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="C44" s="8" t="s">
+      <c r="D44" s="8" t="s">
         <v>156</v>
-      </c>
-      <c r="D44" s="8" t="s">
-        <v>157</v>
       </c>
       <c r="E44" s="7"/>
       <c r="F44" s="7"/>
@@ -2123,10 +2205,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="B45" s="7" t="s">
         <v>158</v>
-      </c>
-      <c r="B45" s="7" t="s">
-        <v>155</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>159</v>
@@ -2144,7 +2226,7 @@
         <v>161</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C46" s="8" t="s">
         <v>162</v>
@@ -2162,7 +2244,7 @@
         <v>164</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>165</v>
@@ -2180,13 +2262,13 @@
         <v>167</v>
       </c>
       <c r="B48" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="C48" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="C48" s="8" t="s">
+      <c r="D48" s="8" t="s">
         <v>169</v>
-      </c>
-      <c r="D48" s="8" t="s">
-        <v>170</v>
       </c>
       <c r="E48" s="7"/>
       <c r="F48" s="7"/>
@@ -2195,10 +2277,10 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="B49" s="7" t="s">
         <v>171</v>
-      </c>
-      <c r="B49" s="7" t="s">
-        <v>168</v>
       </c>
       <c r="C49" s="8" t="s">
         <v>172</v>
@@ -2211,12 +2293,12 @@
       <c r="G49" s="7"/>
       <c r="H49" s="8"/>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
         <v>174</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>175</v>
@@ -2234,7 +2316,7 @@
         <v>177</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C51" s="8" t="s">
         <v>178</v>
@@ -2252,7 +2334,7 @@
         <v>180</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>181</v>
@@ -2265,12 +2347,12 @@
       <c r="G52" s="7"/>
       <c r="H52" s="8"/>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
         <v>183</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C53" s="8" t="s">
         <v>184</v>
@@ -2288,7 +2370,7 @@
         <v>186</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C54" s="8" t="s">
         <v>187</v>
@@ -2301,12 +2383,12 @@
       <c r="G54" s="7"/>
       <c r="H54" s="8"/>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
         <v>189</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C55" s="8" t="s">
         <v>190</v>
@@ -2324,7 +2406,7 @@
         <v>192</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C56" s="8" t="s">
         <v>193</v>
@@ -2396,13 +2478,13 @@
         <v>205</v>
       </c>
       <c r="B60" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="C60" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="C60" s="8" t="s">
+      <c r="D60" s="8" t="s">
         <v>207</v>
-      </c>
-      <c r="D60" s="8" t="s">
-        <v>208</v>
       </c>
       <c r="E60" s="7"/>
       <c r="F60" s="7"/>
@@ -2411,16 +2493,16 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="C61" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="B61" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="C61" s="8" t="s">
+      <c r="D61" s="8" t="s">
         <v>210</v>
-      </c>
-      <c r="D61" s="8" t="s">
-        <v>211</v>
       </c>
       <c r="E61" s="7"/>
       <c r="F61" s="7"/>
@@ -2429,16 +2511,16 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="B62" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="C62" s="8" t="s">
         <v>212</v>
       </c>
-      <c r="B62" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="C62" s="8" t="s">
+      <c r="D62" s="8" t="s">
         <v>213</v>
-      </c>
-      <c r="D62" s="8" t="s">
-        <v>214</v>
       </c>
       <c r="E62" s="7"/>
       <c r="F62" s="7"/>
@@ -2447,16 +2529,16 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="C63" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="B63" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="C63" s="8" t="s">
+      <c r="D63" s="8" t="s">
         <v>216</v>
-      </c>
-      <c r="D63" s="8" t="s">
-        <v>217</v>
       </c>
       <c r="E63" s="7"/>
       <c r="F63" s="7"/>
@@ -2465,16 +2547,16 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="B64" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="C64" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="B64" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="C64" s="8" t="s">
+      <c r="D64" s="8" t="s">
         <v>219</v>
-      </c>
-      <c r="D64" s="8" t="s">
-        <v>220</v>
       </c>
       <c r="E64" s="7"/>
       <c r="F64" s="7"/>
@@ -2483,16 +2565,16 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="B65" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="C65" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="B65" s="7" t="s">
+      <c r="D65" s="8" t="s">
         <v>222</v>
-      </c>
-      <c r="C65" s="8" t="s">
-        <v>223</v>
-      </c>
-      <c r="D65" s="8" t="s">
-        <v>224</v>
       </c>
       <c r="E65" s="7"/>
       <c r="F65" s="7"/>
@@ -2501,16 +2583,16 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="B66" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C66" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="B66" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="C66" s="8" t="s">
+      <c r="D66" s="8" t="s">
         <v>226</v>
-      </c>
-      <c r="D66" s="8" t="s">
-        <v>227</v>
       </c>
       <c r="E66" s="7"/>
       <c r="F66" s="7"/>
@@ -2519,16 +2601,16 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C67" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="B67" s="7" t="s">
+      <c r="D67" s="8" t="s">
         <v>229</v>
-      </c>
-      <c r="C67" s="8" t="s">
-        <v>230</v>
-      </c>
-      <c r="D67" s="8" t="s">
-        <v>231</v>
       </c>
       <c r="E67" s="7"/>
       <c r="F67" s="7"/>
@@ -2537,16 +2619,16 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="B68" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="D68" s="8" t="s">
         <v>232</v>
-      </c>
-      <c r="B68" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="C68" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="D68" s="8" t="s">
-        <v>234</v>
       </c>
       <c r="E68" s="7"/>
       <c r="F68" s="7"/>
@@ -2555,16 +2637,16 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="B69" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C69" s="8" t="s">
         <v>235</v>
       </c>
-      <c r="B69" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="C69" s="8" t="s">
+      <c r="D69" s="8" t="s">
         <v>236</v>
-      </c>
-      <c r="D69" s="8" t="s">
-        <v>234</v>
       </c>
       <c r="E69" s="7"/>
       <c r="F69" s="7"/>
@@ -2576,13 +2658,13 @@
         <v>237</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="C70" s="8" t="s">
         <v>238</v>
       </c>
       <c r="D70" s="8" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="E70" s="7"/>
       <c r="F70" s="7"/>
@@ -2591,26 +2673,188 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="E71" s="7"/>
       <c r="F71" s="7"/>
       <c r="G71" s="7"/>
       <c r="H71" s="8"/>
     </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="B72" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>244</v>
+      </c>
+      <c r="D72" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="E72" s="7"/>
+      <c r="F72" s="7"/>
+      <c r="G72" s="7"/>
+      <c r="H72" s="8"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="B73" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C73" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="D73" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="E73" s="7"/>
+      <c r="F73" s="7"/>
+      <c r="G73" s="7"/>
+      <c r="H73" s="8"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="B74" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="E74" s="7"/>
+      <c r="F74" s="7"/>
+      <c r="G74" s="7"/>
+      <c r="H74" s="8"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="B75" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C75" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="D75" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="E75" s="7"/>
+      <c r="F75" s="7"/>
+      <c r="G75" s="7"/>
+      <c r="H75" s="8"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="B76" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="D76" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="E76" s="7"/>
+      <c r="F76" s="7"/>
+      <c r="G76" s="7"/>
+      <c r="H76" s="8"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="B77" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="C77" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="D77" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="E77" s="7"/>
+      <c r="F77" s="7"/>
+      <c r="G77" s="7"/>
+      <c r="H77" s="8"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="B78" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="D78" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="E78" s="7"/>
+      <c r="F78" s="7"/>
+      <c r="G78" s="7"/>
+      <c r="H78" s="8"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="B79" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="C79" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="D79" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="E79" s="7"/>
+      <c r="F79" s="7"/>
+      <c r="G79" s="7"/>
+      <c r="H79" s="8"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="B80" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="D80" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="E80" s="7"/>
+      <c r="F80" s="7"/>
+      <c r="G80" s="7"/>
+      <c r="H80" s="8"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H71"/>
+  <autoFilter ref="A1:H80"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E71" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E80" type="list">
       <formula1>"Pass,Fail,Blocked,N/A"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Add get_marvis_actions, get_alarms, get_wired_clients + docs/test plan - v1.9.0
</commit_message>
<xml_diff>
--- a/TEST_RESULTS_TRACKER.xlsx
+++ b/TEST_RESULTS_TRACKER.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Test Results" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Results'!$A$1:$H$80</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Results'!$A$1:$H$83</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="278">
   <si>
     <t xml:space="preserve">HPE Networking Assistant — Test Results Summary</t>
   </si>
@@ -143,7 +143,7 @@
     <t xml:space="preserve">Run pytest -q</t>
   </si>
   <si>
-    <t xml:space="preserve">66 passed</t>
+    <t xml:space="preserve">74 passed</t>
   </si>
   <si>
     <t xml:space="preserve">A3</t>
@@ -362,6 +362,33 @@
     <t xml:space="preserve">Numbers match</t>
   </si>
   <si>
+    <t xml:space="preserve">RO-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">get_wired_clients</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wired clients: switch MAC, port, VLAN, IP, vendor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RO-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">get_marvis_actions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marvis actions + fixes; per-category counts; status=open filters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RO-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">get_alarms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alarms with per-severity/per-type counts</t>
+  </si>
+  <si>
     <t xml:space="preserve">RPT-1</t>
   </si>
   <si>
@@ -830,7 +857,7 @@
     <t xml:space="preserve">SC-5</t>
   </si>
   <si>
-    <t xml:space="preserve">Automated suite 66 passed</t>
+    <t xml:space="preserve">Automated suite 74 passed</t>
   </si>
 </sst>
 </file>
@@ -1317,8 +1344,8 @@
         <v>7</v>
       </c>
       <c r="B9" s="3" t="n">
-        <f aca="false">COUNTA('Test Results'!A2:A80)</f>
-        <v>79</v>
+        <f aca="false">COUNTA('Test Results'!A2:A83)</f>
+        <v>82</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1326,7 +1353,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E80,"Pass")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E83,"Pass")</f>
         <v>0</v>
       </c>
     </row>
@@ -1335,7 +1362,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E80,"Fail")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E83,"Fail")</f>
         <v>0</v>
       </c>
     </row>
@@ -1344,7 +1371,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E80,"Blocked")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E83,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
@@ -1353,7 +1380,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E80,"N/A")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E83,"N/A")</f>
         <v>0</v>
       </c>
     </row>
@@ -1363,7 +1390,7 @@
       </c>
       <c r="B14" s="3" t="n">
         <f aca="false">B9-(B10+B11+B12+B13)</f>
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1391,7 +1418,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -1951,36 +1978,36 @@
       <c r="G30" s="7"/>
       <c r="H30" s="8"/>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
         <v>112</v>
       </c>
       <c r="B31" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C31" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="D31" s="8" t="s">
         <v>114</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>115</v>
       </c>
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
       <c r="G31" s="7"/>
       <c r="H31" s="8"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C32" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="B32" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="C32" s="8" t="s">
+      <c r="D32" s="8" t="s">
         <v>117</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>118</v>
       </c>
       <c r="E32" s="7"/>
       <c r="F32" s="7"/>
@@ -1989,16 +2016,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C33" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="B33" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="C33" s="8" t="s">
+      <c r="D33" s="8" t="s">
         <v>120</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>121</v>
       </c>
       <c r="E33" s="7"/>
       <c r="F33" s="7"/>
@@ -2007,10 +2034,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="B34" s="7" t="s">
         <v>122</v>
-      </c>
-      <c r="B34" s="7" t="s">
-        <v>113</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>123</v>
@@ -2028,7 +2055,7 @@
         <v>125</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>126</v>
@@ -2046,13 +2073,13 @@
         <v>128</v>
       </c>
       <c r="B36" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C36" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="C36" s="8" t="s">
+      <c r="D36" s="8" t="s">
         <v>130</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>131</v>
       </c>
       <c r="E36" s="7"/>
       <c r="F36" s="7"/>
@@ -2061,16 +2088,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C37" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="B37" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="C37" s="8" t="s">
+      <c r="D37" s="8" t="s">
         <v>133</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>134</v>
       </c>
       <c r="E37" s="7"/>
       <c r="F37" s="7"/>
@@ -2079,16 +2106,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C38" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="B38" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="C38" s="8" t="s">
+      <c r="D38" s="8" t="s">
         <v>136</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>137</v>
       </c>
       <c r="E38" s="7"/>
       <c r="F38" s="7"/>
@@ -2097,10 +2124,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B39" s="7" t="s">
         <v>138</v>
-      </c>
-      <c r="B39" s="7" t="s">
-        <v>129</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>139</v>
@@ -2118,13 +2145,13 @@
         <v>141</v>
       </c>
       <c r="B40" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="C40" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="C40" s="8" t="s">
+      <c r="D40" s="8" t="s">
         <v>143</v>
-      </c>
-      <c r="D40" s="8" t="s">
-        <v>144</v>
       </c>
       <c r="E40" s="7"/>
       <c r="F40" s="7"/>
@@ -2133,16 +2160,16 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="C41" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="B41" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="C41" s="8" t="s">
+      <c r="D41" s="8" t="s">
         <v>146</v>
-      </c>
-      <c r="D41" s="8" t="s">
-        <v>147</v>
       </c>
       <c r="E41" s="7"/>
       <c r="F41" s="7"/>
@@ -2151,16 +2178,16 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="C42" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="B42" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="C42" s="8" t="s">
+      <c r="D42" s="8" t="s">
         <v>149</v>
-      </c>
-      <c r="D42" s="8" t="s">
-        <v>150</v>
       </c>
       <c r="E42" s="7"/>
       <c r="F42" s="7"/>
@@ -2169,10 +2196,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="B43" s="7" t="s">
         <v>151</v>
-      </c>
-      <c r="B43" s="7" t="s">
-        <v>142</v>
       </c>
       <c r="C43" s="8" t="s">
         <v>152</v>
@@ -2185,12 +2212,12 @@
       <c r="G43" s="7"/>
       <c r="H43" s="8"/>
     </row>
-    <row r="44" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
         <v>154</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>155</v>
@@ -2208,13 +2235,13 @@
         <v>157</v>
       </c>
       <c r="B45" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="C45" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="C45" s="8" t="s">
+      <c r="D45" s="8" t="s">
         <v>159</v>
-      </c>
-      <c r="D45" s="8" t="s">
-        <v>160</v>
       </c>
       <c r="E45" s="7"/>
       <c r="F45" s="7"/>
@@ -2223,34 +2250,34 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="C46" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="B46" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="C46" s="8" t="s">
+      <c r="D46" s="8" t="s">
         <v>162</v>
-      </c>
-      <c r="D46" s="8" t="s">
-        <v>163</v>
       </c>
       <c r="E46" s="7"/>
       <c r="F46" s="7"/>
       <c r="G46" s="7"/>
       <c r="H46" s="8"/>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="C47" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="B47" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="C47" s="8" t="s">
+      <c r="D47" s="8" t="s">
         <v>165</v>
-      </c>
-      <c r="D47" s="8" t="s">
-        <v>166</v>
       </c>
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
@@ -2259,10 +2286,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="B48" s="7" t="s">
         <v>167</v>
-      </c>
-      <c r="B48" s="7" t="s">
-        <v>158</v>
       </c>
       <c r="C48" s="8" t="s">
         <v>168</v>
@@ -2280,31 +2307,31 @@
         <v>170</v>
       </c>
       <c r="B49" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="C49" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C49" s="8" t="s">
+      <c r="D49" s="8" t="s">
         <v>172</v>
-      </c>
-      <c r="D49" s="8" t="s">
-        <v>173</v>
       </c>
       <c r="E49" s="7"/>
       <c r="F49" s="7"/>
       <c r="G49" s="7"/>
       <c r="H49" s="8"/>
     </row>
-    <row r="50" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="C50" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="B50" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="C50" s="8" t="s">
+      <c r="D50" s="8" t="s">
         <v>175</v>
-      </c>
-      <c r="D50" s="8" t="s">
-        <v>176</v>
       </c>
       <c r="E50" s="7"/>
       <c r="F50" s="7"/>
@@ -2313,16 +2340,16 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="C51" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="B51" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="C51" s="8" t="s">
+      <c r="D51" s="8" t="s">
         <v>178</v>
-      </c>
-      <c r="D51" s="8" t="s">
-        <v>179</v>
       </c>
       <c r="E51" s="7"/>
       <c r="F51" s="7"/>
@@ -2331,10 +2358,10 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="B52" s="7" t="s">
         <v>180</v>
-      </c>
-      <c r="B52" s="7" t="s">
-        <v>171</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>181</v>
@@ -2352,7 +2379,7 @@
         <v>183</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="C53" s="8" t="s">
         <v>184</v>
@@ -2370,7 +2397,7 @@
         <v>186</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="C54" s="8" t="s">
         <v>187</v>
@@ -2383,12 +2410,12 @@
       <c r="G54" s="7"/>
       <c r="H54" s="8"/>
     </row>
-    <row r="55" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
         <v>189</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="C55" s="8" t="s">
         <v>190</v>
@@ -2401,12 +2428,12 @@
       <c r="G55" s="7"/>
       <c r="H55" s="8"/>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
         <v>192</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="C56" s="8" t="s">
         <v>193</v>
@@ -2424,31 +2451,31 @@
         <v>195</v>
       </c>
       <c r="B57" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C57" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="C57" s="8" t="s">
+      <c r="D57" s="8" t="s">
         <v>197</v>
-      </c>
-      <c r="D57" s="8" t="s">
-        <v>198</v>
       </c>
       <c r="E57" s="7"/>
       <c r="F57" s="7"/>
       <c r="G57" s="7"/>
       <c r="H57" s="8"/>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C58" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="B58" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="C58" s="8" t="s">
+      <c r="D58" s="8" t="s">
         <v>200</v>
-      </c>
-      <c r="D58" s="8" t="s">
-        <v>201</v>
       </c>
       <c r="E58" s="7"/>
       <c r="F58" s="7"/>
@@ -2457,16 +2484,16 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="B59" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C59" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="B59" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="C59" s="8" t="s">
+      <c r="D59" s="8" t="s">
         <v>203</v>
-      </c>
-      <c r="D59" s="8" t="s">
-        <v>204</v>
       </c>
       <c r="E59" s="7"/>
       <c r="F59" s="7"/>
@@ -2475,10 +2502,10 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="B60" s="7" t="s">
         <v>205</v>
-      </c>
-      <c r="B60" s="7" t="s">
-        <v>196</v>
       </c>
       <c r="C60" s="8" t="s">
         <v>206</v>
@@ -2496,7 +2523,7 @@
         <v>208</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="C61" s="8" t="s">
         <v>209</v>
@@ -2514,7 +2541,7 @@
         <v>211</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="C62" s="8" t="s">
         <v>212</v>
@@ -2532,7 +2559,7 @@
         <v>214</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="C63" s="8" t="s">
         <v>215</v>
@@ -2550,7 +2577,7 @@
         <v>217</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="C64" s="8" t="s">
         <v>218</v>
@@ -2568,7 +2595,7 @@
         <v>220</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="C65" s="8" t="s">
         <v>221</v>
@@ -2586,13 +2613,13 @@
         <v>223</v>
       </c>
       <c r="B66" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="C66" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="C66" s="8" t="s">
+      <c r="D66" s="8" t="s">
         <v>225</v>
-      </c>
-      <c r="D66" s="8" t="s">
-        <v>226</v>
       </c>
       <c r="E66" s="7"/>
       <c r="F66" s="7"/>
@@ -2601,16 +2628,16 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="C67" s="8" t="s">
         <v>227</v>
       </c>
-      <c r="B67" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="C67" s="8" t="s">
+      <c r="D67" s="8" t="s">
         <v>228</v>
-      </c>
-      <c r="D67" s="8" t="s">
-        <v>229</v>
       </c>
       <c r="E67" s="7"/>
       <c r="F67" s="7"/>
@@ -2619,16 +2646,16 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="B68" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="C68" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="B68" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="C68" s="8" t="s">
+      <c r="D68" s="8" t="s">
         <v>231</v>
-      </c>
-      <c r="D68" s="8" t="s">
-        <v>232</v>
       </c>
       <c r="E68" s="7"/>
       <c r="F68" s="7"/>
@@ -2637,16 +2664,16 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="B69" s="7" t="s">
         <v>233</v>
       </c>
-      <c r="B69" s="7" t="s">
+      <c r="C69" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="C69" s="8" t="s">
+      <c r="D69" s="8" t="s">
         <v>235</v>
-      </c>
-      <c r="D69" s="8" t="s">
-        <v>236</v>
       </c>
       <c r="E69" s="7"/>
       <c r="F69" s="7"/>
@@ -2655,16 +2682,16 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="B70" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="C70" s="8" t="s">
         <v>237</v>
       </c>
-      <c r="B70" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="C70" s="8" t="s">
+      <c r="D70" s="8" t="s">
         <v>238</v>
-      </c>
-      <c r="D70" s="8" t="s">
-        <v>239</v>
       </c>
       <c r="E70" s="7"/>
       <c r="F70" s="7"/>
@@ -2673,16 +2700,16 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="B71" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="C71" s="8" t="s">
         <v>240</v>
       </c>
-      <c r="B71" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="C71" s="8" t="s">
+      <c r="D71" s="8" t="s">
         <v>241</v>
-      </c>
-      <c r="D71" s="8" t="s">
-        <v>242</v>
       </c>
       <c r="E71" s="7"/>
       <c r="F71" s="7"/>
@@ -2691,10 +2718,10 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="B72" s="7" t="s">
         <v>243</v>
-      </c>
-      <c r="B72" s="7" t="s">
-        <v>234</v>
       </c>
       <c r="C72" s="8" t="s">
         <v>244</v>
@@ -2712,7 +2739,7 @@
         <v>246</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="C73" s="8" t="s">
         <v>247</v>
@@ -2730,13 +2757,13 @@
         <v>249</v>
       </c>
       <c r="B74" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C74" s="8" t="s">
         <v>250</v>
       </c>
-      <c r="C74" s="8" t="s">
+      <c r="D74" s="8" t="s">
         <v>251</v>
-      </c>
-      <c r="D74" s="8" t="s">
-        <v>252</v>
       </c>
       <c r="E74" s="7"/>
       <c r="F74" s="7"/>
@@ -2745,16 +2772,16 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="B75" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C75" s="8" t="s">
         <v>253</v>
       </c>
-      <c r="B75" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="C75" s="8" t="s">
+      <c r="D75" s="8" t="s">
         <v>254</v>
-      </c>
-      <c r="D75" s="8" t="s">
-        <v>255</v>
       </c>
       <c r="E75" s="7"/>
       <c r="F75" s="7"/>
@@ -2763,16 +2790,16 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="B76" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C76" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="B76" s="7" t="s">
+      <c r="D76" s="8" t="s">
         <v>257</v>
-      </c>
-      <c r="C76" s="8" t="s">
-        <v>258</v>
-      </c>
-      <c r="D76" s="8" t="s">
-        <v>259</v>
       </c>
       <c r="E76" s="7"/>
       <c r="F76" s="7"/>
@@ -2781,16 +2808,16 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="B77" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="C77" s="8" t="s">
         <v>260</v>
       </c>
-      <c r="B77" s="7" t="s">
-        <v>257</v>
-      </c>
-      <c r="C77" s="8" t="s">
+      <c r="D77" s="8" t="s">
         <v>261</v>
-      </c>
-      <c r="D77" s="8" t="s">
-        <v>262</v>
       </c>
       <c r="E77" s="7"/>
       <c r="F77" s="7"/>
@@ -2799,16 +2826,16 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="B78" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="C78" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="B78" s="7" t="s">
-        <v>257</v>
-      </c>
-      <c r="C78" s="8" t="s">
+      <c r="D78" s="8" t="s">
         <v>264</v>
-      </c>
-      <c r="D78" s="8" t="s">
-        <v>262</v>
       </c>
       <c r="E78" s="7"/>
       <c r="F78" s="7"/>
@@ -2820,13 +2847,13 @@
         <v>265</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="C79" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D79" s="8" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="E79" s="7"/>
       <c r="F79" s="7"/>
@@ -2835,26 +2862,80 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="7" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B80" s="7" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="C80" s="8" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D80" s="8" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="E80" s="7"/>
       <c r="F80" s="7"/>
       <c r="G80" s="7"/>
       <c r="H80" s="8"/>
     </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="B81" s="7" t="s">
+        <v>266</v>
+      </c>
+      <c r="C81" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="D81" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="E81" s="7"/>
+      <c r="F81" s="7"/>
+      <c r="G81" s="7"/>
+      <c r="H81" s="8"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="B82" s="7" t="s">
+        <v>266</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="D82" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="E82" s="7"/>
+      <c r="F82" s="7"/>
+      <c r="G82" s="7"/>
+      <c r="H82" s="8"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="B83" s="7" t="s">
+        <v>266</v>
+      </c>
+      <c r="C83" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="D83" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="E83" s="7"/>
+      <c r="F83" s="7"/>
+      <c r="G83" s="7"/>
+      <c r="H83" s="8"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H80"/>
+  <autoFilter ref="A1:H83"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E80" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E83" type="list">
       <formula1>"Pass,Fail,Blocked,N/A"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Add get_sle and get_switch_ports + docs/test plan - v1.10.0
</commit_message>
<xml_diff>
--- a/TEST_RESULTS_TRACKER.xlsx
+++ b/TEST_RESULTS_TRACKER.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Test Results" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Results'!$A$1:$H$83</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Results'!$A$1:$H$85</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="284">
   <si>
     <t xml:space="preserve">HPE Networking Assistant — Test Results Summary</t>
   </si>
@@ -143,7 +143,7 @@
     <t xml:space="preserve">Run pytest -q</t>
   </si>
   <si>
-    <t xml:space="preserve">74 passed</t>
+    <t xml:space="preserve">79 passed</t>
   </si>
   <si>
     <t xml:space="preserve">A3</t>
@@ -389,6 +389,24 @@
     <t xml:space="preserve">Alarms with per-severity/per-type counts</t>
   </si>
   <si>
+    <t xml:space="preserve">RO-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">get_sle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-site SLE metrics as percentages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RO-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">get_switch_ports</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Port link/speed/PoE/neighbor; filter by switch/site/up</t>
+  </si>
+  <si>
     <t xml:space="preserve">RPT-1</t>
   </si>
   <si>
@@ -857,7 +875,7 @@
     <t xml:space="preserve">SC-5</t>
   </si>
   <si>
-    <t xml:space="preserve">Automated suite 74 passed</t>
+    <t xml:space="preserve">Automated suite 79 passed</t>
   </si>
 </sst>
 </file>
@@ -1344,8 +1362,8 @@
         <v>7</v>
       </c>
       <c r="B9" s="3" t="n">
-        <f aca="false">COUNTA('Test Results'!A2:A83)</f>
-        <v>82</v>
+        <f aca="false">COUNTA('Test Results'!A2:A85)</f>
+        <v>84</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1353,7 +1371,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E83,"Pass")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E85,"Pass")</f>
         <v>0</v>
       </c>
     </row>
@@ -1362,7 +1380,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E83,"Fail")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E85,"Fail")</f>
         <v>0</v>
       </c>
     </row>
@@ -1371,7 +1389,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E83,"Blocked")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E85,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
@@ -1380,7 +1398,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E83,"N/A")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E85,"N/A")</f>
         <v>0</v>
       </c>
     </row>
@@ -1390,7 +1408,7 @@
       </c>
       <c r="B14" s="3" t="n">
         <f aca="false">B9-(B10+B11+B12+B13)</f>
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1418,7 +1436,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -2037,31 +2055,31 @@
         <v>121</v>
       </c>
       <c r="B34" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C34" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="C34" s="8" t="s">
+      <c r="D34" s="8" t="s">
         <v>123</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>124</v>
       </c>
       <c r="E34" s="7"/>
       <c r="F34" s="7"/>
       <c r="G34" s="7"/>
       <c r="H34" s="8"/>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C35" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="B35" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="C35" s="8" t="s">
+      <c r="D35" s="8" t="s">
         <v>126</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>127</v>
       </c>
       <c r="E35" s="7"/>
       <c r="F35" s="7"/>
@@ -2070,10 +2088,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B36" s="7" t="s">
         <v>128</v>
-      </c>
-      <c r="B36" s="7" t="s">
-        <v>122</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>129</v>
@@ -2091,7 +2109,7 @@
         <v>131</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>132</v>
@@ -2109,7 +2127,7 @@
         <v>134</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>135</v>
@@ -2127,13 +2145,13 @@
         <v>137</v>
       </c>
       <c r="B39" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="C39" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="C39" s="8" t="s">
+      <c r="D39" s="8" t="s">
         <v>139</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>140</v>
       </c>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
@@ -2142,16 +2160,16 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="C40" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B40" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="C40" s="8" t="s">
+      <c r="D40" s="8" t="s">
         <v>142</v>
-      </c>
-      <c r="D40" s="8" t="s">
-        <v>143</v>
       </c>
       <c r="E40" s="7"/>
       <c r="F40" s="7"/>
@@ -2160,10 +2178,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="B41" s="7" t="s">
         <v>144</v>
-      </c>
-      <c r="B41" s="7" t="s">
-        <v>138</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>145</v>
@@ -2181,7 +2199,7 @@
         <v>147</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="C42" s="8" t="s">
         <v>148</v>
@@ -2199,13 +2217,13 @@
         <v>150</v>
       </c>
       <c r="B43" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C43" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="C43" s="8" t="s">
+      <c r="D43" s="8" t="s">
         <v>152</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>153</v>
       </c>
       <c r="E43" s="7"/>
       <c r="F43" s="7"/>
@@ -2214,16 +2232,16 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C44" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="B44" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="C44" s="8" t="s">
+      <c r="D44" s="8" t="s">
         <v>155</v>
-      </c>
-      <c r="D44" s="8" t="s">
-        <v>156</v>
       </c>
       <c r="E44" s="7"/>
       <c r="F44" s="7"/>
@@ -2232,10 +2250,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="B45" s="7" t="s">
         <v>157</v>
-      </c>
-      <c r="B45" s="7" t="s">
-        <v>151</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>158</v>
@@ -2253,7 +2271,7 @@
         <v>160</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C46" s="8" t="s">
         <v>161</v>
@@ -2266,12 +2284,12 @@
       <c r="G46" s="7"/>
       <c r="H46" s="8"/>
     </row>
-    <row r="47" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
         <v>163</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>164</v>
@@ -2289,31 +2307,31 @@
         <v>166</v>
       </c>
       <c r="B48" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="C48" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="C48" s="8" t="s">
+      <c r="D48" s="8" t="s">
         <v>168</v>
-      </c>
-      <c r="D48" s="8" t="s">
-        <v>169</v>
       </c>
       <c r="E48" s="7"/>
       <c r="F48" s="7"/>
       <c r="G48" s="7"/>
       <c r="H48" s="8"/>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="C49" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="B49" s="7" t="s">
-        <v>167</v>
-      </c>
-      <c r="C49" s="8" t="s">
+      <c r="D49" s="8" t="s">
         <v>171</v>
-      </c>
-      <c r="D49" s="8" t="s">
-        <v>172</v>
       </c>
       <c r="E49" s="7"/>
       <c r="F49" s="7"/>
@@ -2322,10 +2340,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="B50" s="7" t="s">
         <v>173</v>
-      </c>
-      <c r="B50" s="7" t="s">
-        <v>167</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>174</v>
@@ -2343,7 +2361,7 @@
         <v>176</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="C51" s="8" t="s">
         <v>177</v>
@@ -2361,31 +2379,31 @@
         <v>179</v>
       </c>
       <c r="B52" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="C52" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="C52" s="8" t="s">
+      <c r="D52" s="8" t="s">
         <v>181</v>
-      </c>
-      <c r="D52" s="8" t="s">
-        <v>182</v>
       </c>
       <c r="E52" s="7"/>
       <c r="F52" s="7"/>
       <c r="G52" s="7"/>
       <c r="H52" s="8"/>
     </row>
-    <row r="53" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="C53" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="B53" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="C53" s="8" t="s">
+      <c r="D53" s="8" t="s">
         <v>184</v>
-      </c>
-      <c r="D53" s="8" t="s">
-        <v>185</v>
       </c>
       <c r="E53" s="7"/>
       <c r="F53" s="7"/>
@@ -2394,10 +2412,10 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="B54" s="7" t="s">
         <v>186</v>
-      </c>
-      <c r="B54" s="7" t="s">
-        <v>180</v>
       </c>
       <c r="C54" s="8" t="s">
         <v>187</v>
@@ -2410,12 +2428,12 @@
       <c r="G54" s="7"/>
       <c r="H54" s="8"/>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
         <v>189</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="C55" s="8" t="s">
         <v>190</v>
@@ -2428,12 +2446,12 @@
       <c r="G55" s="7"/>
       <c r="H55" s="8"/>
     </row>
-    <row r="56" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
         <v>192</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="C56" s="8" t="s">
         <v>193</v>
@@ -2451,7 +2469,7 @@
         <v>195</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="C57" s="8" t="s">
         <v>196</v>
@@ -2469,7 +2487,7 @@
         <v>198</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="C58" s="8" t="s">
         <v>199</v>
@@ -2487,7 +2505,7 @@
         <v>201</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="C59" s="8" t="s">
         <v>202</v>
@@ -2500,18 +2518,18 @@
       <c r="G59" s="7"/>
       <c r="H59" s="8"/>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
         <v>204</v>
       </c>
       <c r="B60" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="C60" s="8" t="s">
         <v>205</v>
       </c>
-      <c r="C60" s="8" t="s">
+      <c r="D60" s="8" t="s">
         <v>206</v>
-      </c>
-      <c r="D60" s="8" t="s">
-        <v>207</v>
       </c>
       <c r="E60" s="7"/>
       <c r="F60" s="7"/>
@@ -2520,16 +2538,16 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="C61" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="B61" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="C61" s="8" t="s">
+      <c r="D61" s="8" t="s">
         <v>209</v>
-      </c>
-      <c r="D61" s="8" t="s">
-        <v>210</v>
       </c>
       <c r="E61" s="7"/>
       <c r="F61" s="7"/>
@@ -2538,10 +2556,10 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="B62" s="7" t="s">
         <v>211</v>
-      </c>
-      <c r="B62" s="7" t="s">
-        <v>205</v>
       </c>
       <c r="C62" s="8" t="s">
         <v>212</v>
@@ -2559,7 +2577,7 @@
         <v>214</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="C63" s="8" t="s">
         <v>215</v>
@@ -2577,7 +2595,7 @@
         <v>217</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="C64" s="8" t="s">
         <v>218</v>
@@ -2595,7 +2613,7 @@
         <v>220</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="C65" s="8" t="s">
         <v>221</v>
@@ -2613,7 +2631,7 @@
         <v>223</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="C66" s="8" t="s">
         <v>224</v>
@@ -2631,7 +2649,7 @@
         <v>226</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="C67" s="8" t="s">
         <v>227</v>
@@ -2649,7 +2667,7 @@
         <v>229</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="C68" s="8" t="s">
         <v>230</v>
@@ -2667,13 +2685,13 @@
         <v>232</v>
       </c>
       <c r="B69" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="C69" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="C69" s="8" t="s">
+      <c r="D69" s="8" t="s">
         <v>234</v>
-      </c>
-      <c r="D69" s="8" t="s">
-        <v>235</v>
       </c>
       <c r="E69" s="7"/>
       <c r="F69" s="7"/>
@@ -2682,16 +2700,16 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="B70" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="C70" s="8" t="s">
         <v>236</v>
       </c>
-      <c r="B70" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="C70" s="8" t="s">
+      <c r="D70" s="8" t="s">
         <v>237</v>
-      </c>
-      <c r="D70" s="8" t="s">
-        <v>238</v>
       </c>
       <c r="E70" s="7"/>
       <c r="F70" s="7"/>
@@ -2700,10 +2718,10 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="B71" s="7" t="s">
         <v>239</v>
-      </c>
-      <c r="B71" s="7" t="s">
-        <v>233</v>
       </c>
       <c r="C71" s="8" t="s">
         <v>240</v>
@@ -2721,13 +2739,13 @@
         <v>242</v>
       </c>
       <c r="B72" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="C72" s="8" t="s">
         <v>243</v>
       </c>
-      <c r="C72" s="8" t="s">
+      <c r="D72" s="8" t="s">
         <v>244</v>
-      </c>
-      <c r="D72" s="8" t="s">
-        <v>245</v>
       </c>
       <c r="E72" s="7"/>
       <c r="F72" s="7"/>
@@ -2736,16 +2754,16 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="B73" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="C73" s="8" t="s">
         <v>246</v>
       </c>
-      <c r="B73" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="C73" s="8" t="s">
+      <c r="D73" s="8" t="s">
         <v>247</v>
-      </c>
-      <c r="D73" s="8" t="s">
-        <v>248</v>
       </c>
       <c r="E73" s="7"/>
       <c r="F73" s="7"/>
@@ -2754,10 +2772,10 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="B74" s="7" t="s">
         <v>249</v>
-      </c>
-      <c r="B74" s="7" t="s">
-        <v>243</v>
       </c>
       <c r="C74" s="8" t="s">
         <v>250</v>
@@ -2775,7 +2793,7 @@
         <v>252</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="C75" s="8" t="s">
         <v>253</v>
@@ -2793,7 +2811,7 @@
         <v>255</v>
       </c>
       <c r="B76" s="7" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="C76" s="8" t="s">
         <v>256</v>
@@ -2811,13 +2829,13 @@
         <v>258</v>
       </c>
       <c r="B77" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="C77" s="8" t="s">
         <v>259</v>
       </c>
-      <c r="C77" s="8" t="s">
+      <c r="D77" s="8" t="s">
         <v>260</v>
-      </c>
-      <c r="D77" s="8" t="s">
-        <v>261</v>
       </c>
       <c r="E77" s="7"/>
       <c r="F77" s="7"/>
@@ -2826,16 +2844,16 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="B78" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="C78" s="8" t="s">
         <v>262</v>
       </c>
-      <c r="B78" s="7" t="s">
-        <v>259</v>
-      </c>
-      <c r="C78" s="8" t="s">
+      <c r="D78" s="8" t="s">
         <v>263</v>
-      </c>
-      <c r="D78" s="8" t="s">
-        <v>264</v>
       </c>
       <c r="E78" s="7"/>
       <c r="F78" s="7"/>
@@ -2844,16 +2862,16 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="7" t="s">
+        <v>264</v>
+      </c>
+      <c r="B79" s="7" t="s">
         <v>265</v>
       </c>
-      <c r="B79" s="7" t="s">
+      <c r="C79" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="C79" s="8" t="s">
+      <c r="D79" s="8" t="s">
         <v>267</v>
-      </c>
-      <c r="D79" s="8" t="s">
-        <v>268</v>
       </c>
       <c r="E79" s="7"/>
       <c r="F79" s="7"/>
@@ -2862,16 +2880,16 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="B80" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="C80" s="8" t="s">
         <v>269</v>
       </c>
-      <c r="B80" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="C80" s="8" t="s">
+      <c r="D80" s="8" t="s">
         <v>270</v>
-      </c>
-      <c r="D80" s="8" t="s">
-        <v>271</v>
       </c>
       <c r="E80" s="7"/>
       <c r="F80" s="7"/>
@@ -2880,16 +2898,16 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="B81" s="7" t="s">
         <v>272</v>
-      </c>
-      <c r="B81" s="7" t="s">
-        <v>266</v>
       </c>
       <c r="C81" s="8" t="s">
         <v>273</v>
       </c>
       <c r="D81" s="8" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="E81" s="7"/>
       <c r="F81" s="7"/>
@@ -2898,16 +2916,16 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B82" s="7" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="C82" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D82" s="8" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="E82" s="7"/>
       <c r="F82" s="7"/>
@@ -2916,26 +2934,62 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="7" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B83" s="7" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="C83" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="D83" s="8" t="s">
         <v>277</v>
-      </c>
-      <c r="D83" s="8" t="s">
-        <v>271</v>
       </c>
       <c r="E83" s="7"/>
       <c r="F83" s="7"/>
       <c r="G83" s="7"/>
       <c r="H83" s="8"/>
     </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="B84" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="D84" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="E84" s="7"/>
+      <c r="F84" s="7"/>
+      <c r="G84" s="7"/>
+      <c r="H84" s="8"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="B85" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="C85" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="D85" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="E85" s="7"/>
+      <c r="F85" s="7"/>
+      <c r="G85" s="7"/>
+      <c r="H85" s="8"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H83"/>
+  <autoFilter ref="A1:H85"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E83" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E85" type="list">
       <formula1>"Pass,Fail,Blocked,N/A"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Add export_org_config (org config backup) + docs - v1.11.0
</commit_message>
<xml_diff>
--- a/TEST_RESULTS_TRACKER.xlsx
+++ b/TEST_RESULTS_TRACKER.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Test Results" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Results'!$A$1:$H$85</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Results'!$A$1:$H$86</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="287">
   <si>
     <t xml:space="preserve">HPE Networking Assistant — Test Results Summary</t>
   </si>
@@ -143,7 +143,7 @@
     <t xml:space="preserve">Run pytest -q</t>
   </si>
   <si>
-    <t xml:space="preserve">79 passed</t>
+    <t xml:space="preserve">82 passed</t>
   </si>
   <si>
     <t xml:space="preserve">A3</t>
@@ -407,6 +407,15 @@
     <t xml:space="preserve">Port link/speed/PoE/neighbor; filter by switch/site/up</t>
   </si>
   <si>
+    <t xml:space="preserve">RO-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">export_org_config</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JSON config backup (org+sites/networks/templates/WLANs/NAC); per-type counts</t>
+  </si>
+  <si>
     <t xml:space="preserve">RPT-1</t>
   </si>
   <si>
@@ -875,7 +884,7 @@
     <t xml:space="preserve">SC-5</t>
   </si>
   <si>
-    <t xml:space="preserve">Automated suite 79 passed</t>
+    <t xml:space="preserve">Automated suite 82 passed</t>
   </si>
 </sst>
 </file>
@@ -1362,8 +1371,8 @@
         <v>7</v>
       </c>
       <c r="B9" s="3" t="n">
-        <f aca="false">COUNTA('Test Results'!A2:A85)</f>
-        <v>84</v>
+        <f aca="false">COUNTA('Test Results'!A2:A86)</f>
+        <v>85</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1371,7 +1380,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E85,"Pass")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E86,"Pass")</f>
         <v>0</v>
       </c>
     </row>
@@ -1380,7 +1389,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E85,"Fail")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E86,"Fail")</f>
         <v>0</v>
       </c>
     </row>
@@ -1389,7 +1398,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E85,"Blocked")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E86,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
@@ -1398,7 +1407,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E85,"N/A")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E86,"N/A")</f>
         <v>0</v>
       </c>
     </row>
@@ -1408,7 +1417,7 @@
       </c>
       <c r="B14" s="3" t="n">
         <f aca="false">B9-(B10+B11+B12+B13)</f>
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1436,7 +1445,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -2086,18 +2095,18 @@
       <c r="G35" s="7"/>
       <c r="H35" s="8"/>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
         <v>127</v>
       </c>
       <c r="B36" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C36" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="C36" s="8" t="s">
+      <c r="D36" s="8" t="s">
         <v>129</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>130</v>
       </c>
       <c r="E36" s="7"/>
       <c r="F36" s="7"/>
@@ -2106,10 +2115,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B37" s="7" t="s">
         <v>131</v>
-      </c>
-      <c r="B37" s="7" t="s">
-        <v>128</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>132</v>
@@ -2127,7 +2136,7 @@
         <v>134</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>135</v>
@@ -2145,7 +2154,7 @@
         <v>137</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>138</v>
@@ -2163,7 +2172,7 @@
         <v>140</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>141</v>
@@ -2181,13 +2190,13 @@
         <v>143</v>
       </c>
       <c r="B41" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="C41" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="C41" s="8" t="s">
+      <c r="D41" s="8" t="s">
         <v>145</v>
-      </c>
-      <c r="D41" s="8" t="s">
-        <v>146</v>
       </c>
       <c r="E41" s="7"/>
       <c r="F41" s="7"/>
@@ -2196,10 +2205,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="B42" s="7" t="s">
         <v>147</v>
-      </c>
-      <c r="B42" s="7" t="s">
-        <v>144</v>
       </c>
       <c r="C42" s="8" t="s">
         <v>148</v>
@@ -2217,7 +2226,7 @@
         <v>150</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C43" s="8" t="s">
         <v>151</v>
@@ -2235,7 +2244,7 @@
         <v>153</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>154</v>
@@ -2253,13 +2262,13 @@
         <v>156</v>
       </c>
       <c r="B45" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="C45" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C45" s="8" t="s">
+      <c r="D45" s="8" t="s">
         <v>158</v>
-      </c>
-      <c r="D45" s="8" t="s">
-        <v>159</v>
       </c>
       <c r="E45" s="7"/>
       <c r="F45" s="7"/>
@@ -2268,10 +2277,10 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="B46" s="7" t="s">
         <v>160</v>
-      </c>
-      <c r="B46" s="7" t="s">
-        <v>157</v>
       </c>
       <c r="C46" s="8" t="s">
         <v>161</v>
@@ -2289,7 +2298,7 @@
         <v>163</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>164</v>
@@ -2307,7 +2316,7 @@
         <v>166</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C48" s="8" t="s">
         <v>167</v>
@@ -2320,12 +2329,12 @@
       <c r="G48" s="7"/>
       <c r="H48" s="8"/>
     </row>
-    <row r="49" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
         <v>169</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C49" s="8" t="s">
         <v>170</v>
@@ -2338,18 +2347,18 @@
       <c r="G49" s="7"/>
       <c r="H49" s="8"/>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
         <v>172</v>
       </c>
       <c r="B50" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="C50" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="C50" s="8" t="s">
+      <c r="D50" s="8" t="s">
         <v>174</v>
-      </c>
-      <c r="D50" s="8" t="s">
-        <v>175</v>
       </c>
       <c r="E50" s="7"/>
       <c r="F50" s="7"/>
@@ -2358,10 +2367,10 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="B51" s="7" t="s">
         <v>176</v>
-      </c>
-      <c r="B51" s="7" t="s">
-        <v>173</v>
       </c>
       <c r="C51" s="8" t="s">
         <v>177</v>
@@ -2379,7 +2388,7 @@
         <v>179</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>180</v>
@@ -2397,7 +2406,7 @@
         <v>182</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C53" s="8" t="s">
         <v>183</v>
@@ -2415,25 +2424,25 @@
         <v>185</v>
       </c>
       <c r="B54" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="C54" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="C54" s="8" t="s">
+      <c r="D54" s="8" t="s">
         <v>187</v>
-      </c>
-      <c r="D54" s="8" t="s">
-        <v>188</v>
       </c>
       <c r="E54" s="7"/>
       <c r="F54" s="7"/>
       <c r="G54" s="7"/>
       <c r="H54" s="8"/>
     </row>
-    <row r="55" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="B55" s="7" t="s">
         <v>189</v>
-      </c>
-      <c r="B55" s="7" t="s">
-        <v>186</v>
       </c>
       <c r="C55" s="8" t="s">
         <v>190</v>
@@ -2446,12 +2455,12 @@
       <c r="G55" s="7"/>
       <c r="H55" s="8"/>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
         <v>192</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C56" s="8" t="s">
         <v>193</v>
@@ -2469,7 +2478,7 @@
         <v>195</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C57" s="8" t="s">
         <v>196</v>
@@ -2482,12 +2491,12 @@
       <c r="G57" s="7"/>
       <c r="H57" s="8"/>
     </row>
-    <row r="58" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
         <v>198</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C58" s="8" t="s">
         <v>199</v>
@@ -2500,12 +2509,12 @@
       <c r="G58" s="7"/>
       <c r="H58" s="8"/>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
         <v>201</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C59" s="8" t="s">
         <v>202</v>
@@ -2518,12 +2527,12 @@
       <c r="G59" s="7"/>
       <c r="H59" s="8"/>
     </row>
-    <row r="60" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
         <v>204</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C60" s="8" t="s">
         <v>205</v>
@@ -2536,12 +2545,12 @@
       <c r="G60" s="7"/>
       <c r="H60" s="8"/>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
         <v>207</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C61" s="8" t="s">
         <v>208</v>
@@ -2559,13 +2568,13 @@
         <v>210</v>
       </c>
       <c r="B62" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="C62" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="C62" s="8" t="s">
+      <c r="D62" s="8" t="s">
         <v>212</v>
-      </c>
-      <c r="D62" s="8" t="s">
-        <v>213</v>
       </c>
       <c r="E62" s="7"/>
       <c r="F62" s="7"/>
@@ -2574,10 +2583,10 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="B63" s="7" t="s">
         <v>214</v>
-      </c>
-      <c r="B63" s="7" t="s">
-        <v>211</v>
       </c>
       <c r="C63" s="8" t="s">
         <v>215</v>
@@ -2595,7 +2604,7 @@
         <v>217</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C64" s="8" t="s">
         <v>218</v>
@@ -2613,7 +2622,7 @@
         <v>220</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C65" s="8" t="s">
         <v>221</v>
@@ -2631,7 +2640,7 @@
         <v>223</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C66" s="8" t="s">
         <v>224</v>
@@ -2649,7 +2658,7 @@
         <v>226</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C67" s="8" t="s">
         <v>227</v>
@@ -2667,7 +2676,7 @@
         <v>229</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C68" s="8" t="s">
         <v>230</v>
@@ -2685,7 +2694,7 @@
         <v>232</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C69" s="8" t="s">
         <v>233</v>
@@ -2703,7 +2712,7 @@
         <v>235</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C70" s="8" t="s">
         <v>236</v>
@@ -2721,13 +2730,13 @@
         <v>238</v>
       </c>
       <c r="B71" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="C71" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="C71" s="8" t="s">
+      <c r="D71" s="8" t="s">
         <v>240</v>
-      </c>
-      <c r="D71" s="8" t="s">
-        <v>241</v>
       </c>
       <c r="E71" s="7"/>
       <c r="F71" s="7"/>
@@ -2736,10 +2745,10 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="B72" s="7" t="s">
         <v>242</v>
-      </c>
-      <c r="B72" s="7" t="s">
-        <v>239</v>
       </c>
       <c r="C72" s="8" t="s">
         <v>243</v>
@@ -2757,7 +2766,7 @@
         <v>245</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="C73" s="8" t="s">
         <v>246</v>
@@ -2775,13 +2784,13 @@
         <v>248</v>
       </c>
       <c r="B74" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="C74" s="8" t="s">
         <v>249</v>
       </c>
-      <c r="C74" s="8" t="s">
+      <c r="D74" s="8" t="s">
         <v>250</v>
-      </c>
-      <c r="D74" s="8" t="s">
-        <v>251</v>
       </c>
       <c r="E74" s="7"/>
       <c r="F74" s="7"/>
@@ -2790,10 +2799,10 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="B75" s="7" t="s">
         <v>252</v>
-      </c>
-      <c r="B75" s="7" t="s">
-        <v>249</v>
       </c>
       <c r="C75" s="8" t="s">
         <v>253</v>
@@ -2811,7 +2820,7 @@
         <v>255</v>
       </c>
       <c r="B76" s="7" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C76" s="8" t="s">
         <v>256</v>
@@ -2829,7 +2838,7 @@
         <v>258</v>
       </c>
       <c r="B77" s="7" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C77" s="8" t="s">
         <v>259</v>
@@ -2847,7 +2856,7 @@
         <v>261</v>
       </c>
       <c r="B78" s="7" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C78" s="8" t="s">
         <v>262</v>
@@ -2865,13 +2874,13 @@
         <v>264</v>
       </c>
       <c r="B79" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="C79" s="8" t="s">
         <v>265</v>
       </c>
-      <c r="C79" s="8" t="s">
+      <c r="D79" s="8" t="s">
         <v>266</v>
-      </c>
-      <c r="D79" s="8" t="s">
-        <v>267</v>
       </c>
       <c r="E79" s="7"/>
       <c r="F79" s="7"/>
@@ -2880,10 +2889,10 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="B80" s="7" t="s">
         <v>268</v>
-      </c>
-      <c r="B80" s="7" t="s">
-        <v>265</v>
       </c>
       <c r="C80" s="8" t="s">
         <v>269</v>
@@ -2901,13 +2910,13 @@
         <v>271</v>
       </c>
       <c r="B81" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="C81" s="8" t="s">
         <v>272</v>
       </c>
-      <c r="C81" s="8" t="s">
+      <c r="D81" s="8" t="s">
         <v>273</v>
-      </c>
-      <c r="D81" s="8" t="s">
-        <v>274</v>
       </c>
       <c r="E81" s="7"/>
       <c r="F81" s="7"/>
@@ -2916,10 +2925,10 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="B82" s="7" t="s">
         <v>275</v>
-      </c>
-      <c r="B82" s="7" t="s">
-        <v>272</v>
       </c>
       <c r="C82" s="8" t="s">
         <v>276</v>
@@ -2937,13 +2946,13 @@
         <v>278</v>
       </c>
       <c r="B83" s="7" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C83" s="8" t="s">
         <v>279</v>
       </c>
       <c r="D83" s="8" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="E83" s="7"/>
       <c r="F83" s="7"/>
@@ -2952,16 +2961,16 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="B84" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="D84" s="8" t="s">
         <v>280</v>
-      </c>
-      <c r="B84" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="C84" s="8" t="s">
-        <v>281</v>
-      </c>
-      <c r="D84" s="8" t="s">
-        <v>277</v>
       </c>
       <c r="E84" s="7"/>
       <c r="F84" s="7"/>
@@ -2970,26 +2979,44 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="7" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B85" s="7" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C85" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D85" s="8" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="E85" s="7"/>
       <c r="F85" s="7"/>
       <c r="G85" s="7"/>
       <c r="H85" s="8"/>
     </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="B86" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="E86" s="7"/>
+      <c r="F86" s="7"/>
+      <c r="G86" s="7"/>
+      <c r="H86" s="8"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H85"/>
+  <autoFilter ref="A1:H86"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E85" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E86" type="list">
       <formula1>"Pass,Fail,Blocked,N/A"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Add set_active_org (multi-org) and diff_org_config (config drift) + docs - v1.12.0
</commit_message>
<xml_diff>
--- a/TEST_RESULTS_TRACKER.xlsx
+++ b/TEST_RESULTS_TRACKER.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Test Results" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Results'!$A$1:$H$86</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Results'!$A$1:$H$88</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="293">
   <si>
     <t xml:space="preserve">HPE Networking Assistant — Test Results Summary</t>
   </si>
@@ -143,7 +143,7 @@
     <t xml:space="preserve">Run pytest -q</t>
   </si>
   <si>
-    <t xml:space="preserve">82 passed</t>
+    <t xml:space="preserve">87 passed</t>
   </si>
   <si>
     <t xml:space="preserve">A3</t>
@@ -416,6 +416,24 @@
     <t xml:space="preserve">JSON config backup (org+sites/networks/templates/WLANs/NAC); per-type counts</t>
   </si>
   <si>
+    <t xml:space="preserve">RO-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">set_active_org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active org set by name; later tools target it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RO-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">diff_org_config</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Added/removed/changed per resource type vs saved backup</t>
+  </si>
+  <si>
     <t xml:space="preserve">RPT-1</t>
   </si>
   <si>
@@ -884,7 +902,7 @@
     <t xml:space="preserve">SC-5</t>
   </si>
   <si>
-    <t xml:space="preserve">Automated suite 82 passed</t>
+    <t xml:space="preserve">Automated suite 87 passed</t>
   </si>
 </sst>
 </file>
@@ -1371,8 +1389,8 @@
         <v>7</v>
       </c>
       <c r="B9" s="3" t="n">
-        <f aca="false">COUNTA('Test Results'!A2:A86)</f>
-        <v>85</v>
+        <f aca="false">COUNTA('Test Results'!A2:A88)</f>
+        <v>87</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1380,7 +1398,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E86,"Pass")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E88,"Pass")</f>
         <v>0</v>
       </c>
     </row>
@@ -1389,7 +1407,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E86,"Fail")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E88,"Fail")</f>
         <v>0</v>
       </c>
     </row>
@@ -1398,7 +1416,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E86,"Blocked")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E88,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
@@ -1407,7 +1425,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E86,"N/A")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E88,"N/A")</f>
         <v>0</v>
       </c>
     </row>
@@ -1417,7 +1435,7 @@
       </c>
       <c r="B14" s="3" t="n">
         <f aca="false">B9-(B10+B11+B12+B13)</f>
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1445,7 +1463,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -2118,31 +2136,31 @@
         <v>130</v>
       </c>
       <c r="B37" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C37" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="C37" s="8" t="s">
+      <c r="D37" s="8" t="s">
         <v>132</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>133</v>
       </c>
       <c r="E37" s="7"/>
       <c r="F37" s="7"/>
       <c r="G37" s="7"/>
       <c r="H37" s="8"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C38" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="B38" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="C38" s="8" t="s">
+      <c r="D38" s="8" t="s">
         <v>135</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>136</v>
       </c>
       <c r="E38" s="7"/>
       <c r="F38" s="7"/>
@@ -2151,10 +2169,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="B39" s="7" t="s">
         <v>137</v>
-      </c>
-      <c r="B39" s="7" t="s">
-        <v>131</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>138</v>
@@ -2172,7 +2190,7 @@
         <v>140</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>141</v>
@@ -2190,7 +2208,7 @@
         <v>143</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>144</v>
@@ -2208,13 +2226,13 @@
         <v>146</v>
       </c>
       <c r="B42" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="C42" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="C42" s="8" t="s">
+      <c r="D42" s="8" t="s">
         <v>148</v>
-      </c>
-      <c r="D42" s="8" t="s">
-        <v>149</v>
       </c>
       <c r="E42" s="7"/>
       <c r="F42" s="7"/>
@@ -2223,16 +2241,16 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="C43" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="B43" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="C43" s="8" t="s">
+      <c r="D43" s="8" t="s">
         <v>151</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>152</v>
       </c>
       <c r="E43" s="7"/>
       <c r="F43" s="7"/>
@@ -2241,10 +2259,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B44" s="7" t="s">
         <v>153</v>
-      </c>
-      <c r="B44" s="7" t="s">
-        <v>147</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>154</v>
@@ -2262,7 +2280,7 @@
         <v>156</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>157</v>
@@ -2280,13 +2298,13 @@
         <v>159</v>
       </c>
       <c r="B46" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="C46" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="C46" s="8" t="s">
+      <c r="D46" s="8" t="s">
         <v>161</v>
-      </c>
-      <c r="D46" s="8" t="s">
-        <v>162</v>
       </c>
       <c r="E46" s="7"/>
       <c r="F46" s="7"/>
@@ -2295,16 +2313,16 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="C47" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="B47" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="C47" s="8" t="s">
+      <c r="D47" s="8" t="s">
         <v>164</v>
-      </c>
-      <c r="D47" s="8" t="s">
-        <v>165</v>
       </c>
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
@@ -2313,10 +2331,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="B48" s="7" t="s">
         <v>166</v>
-      </c>
-      <c r="B48" s="7" t="s">
-        <v>160</v>
       </c>
       <c r="C48" s="8" t="s">
         <v>167</v>
@@ -2334,7 +2352,7 @@
         <v>169</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="C49" s="8" t="s">
         <v>170</v>
@@ -2347,12 +2365,12 @@
       <c r="G49" s="7"/>
       <c r="H49" s="8"/>
     </row>
-    <row r="50" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
         <v>172</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>173</v>
@@ -2370,31 +2388,31 @@
         <v>175</v>
       </c>
       <c r="B51" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="C51" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C51" s="8" t="s">
+      <c r="D51" s="8" t="s">
         <v>177</v>
-      </c>
-      <c r="D51" s="8" t="s">
-        <v>178</v>
       </c>
       <c r="E51" s="7"/>
       <c r="F51" s="7"/>
       <c r="G51" s="7"/>
       <c r="H51" s="8"/>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="C52" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="B52" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="C52" s="8" t="s">
+      <c r="D52" s="8" t="s">
         <v>180</v>
-      </c>
-      <c r="D52" s="8" t="s">
-        <v>181</v>
       </c>
       <c r="E52" s="7"/>
       <c r="F52" s="7"/>
@@ -2403,10 +2421,10 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="B53" s="7" t="s">
         <v>182</v>
-      </c>
-      <c r="B53" s="7" t="s">
-        <v>176</v>
       </c>
       <c r="C53" s="8" t="s">
         <v>183</v>
@@ -2424,7 +2442,7 @@
         <v>185</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="C54" s="8" t="s">
         <v>186</v>
@@ -2442,31 +2460,31 @@
         <v>188</v>
       </c>
       <c r="B55" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="C55" s="8" t="s">
         <v>189</v>
       </c>
-      <c r="C55" s="8" t="s">
+      <c r="D55" s="8" t="s">
         <v>190</v>
-      </c>
-      <c r="D55" s="8" t="s">
-        <v>191</v>
       </c>
       <c r="E55" s="7"/>
       <c r="F55" s="7"/>
       <c r="G55" s="7"/>
       <c r="H55" s="8"/>
     </row>
-    <row r="56" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="C56" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="B56" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="C56" s="8" t="s">
+      <c r="D56" s="8" t="s">
         <v>193</v>
-      </c>
-      <c r="D56" s="8" t="s">
-        <v>194</v>
       </c>
       <c r="E56" s="7"/>
       <c r="F56" s="7"/>
@@ -2475,10 +2493,10 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="B57" s="7" t="s">
         <v>195</v>
-      </c>
-      <c r="B57" s="7" t="s">
-        <v>189</v>
       </c>
       <c r="C57" s="8" t="s">
         <v>196</v>
@@ -2491,12 +2509,12 @@
       <c r="G57" s="7"/>
       <c r="H57" s="8"/>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
         <v>198</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="C58" s="8" t="s">
         <v>199</v>
@@ -2509,12 +2527,12 @@
       <c r="G58" s="7"/>
       <c r="H58" s="8"/>
     </row>
-    <row r="59" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
         <v>201</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="C59" s="8" t="s">
         <v>202</v>
@@ -2532,7 +2550,7 @@
         <v>204</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="C60" s="8" t="s">
         <v>205</v>
@@ -2550,7 +2568,7 @@
         <v>207</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="C61" s="8" t="s">
         <v>208</v>
@@ -2568,7 +2586,7 @@
         <v>210</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="C62" s="8" t="s">
         <v>211</v>
@@ -2581,18 +2599,18 @@
       <c r="G62" s="7"/>
       <c r="H62" s="8"/>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
         <v>213</v>
       </c>
       <c r="B63" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="C63" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="C63" s="8" t="s">
+      <c r="D63" s="8" t="s">
         <v>215</v>
-      </c>
-      <c r="D63" s="8" t="s">
-        <v>216</v>
       </c>
       <c r="E63" s="7"/>
       <c r="F63" s="7"/>
@@ -2601,16 +2619,16 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="B64" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="C64" s="8" t="s">
         <v>217</v>
       </c>
-      <c r="B64" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="C64" s="8" t="s">
+      <c r="D64" s="8" t="s">
         <v>218</v>
-      </c>
-      <c r="D64" s="8" t="s">
-        <v>219</v>
       </c>
       <c r="E64" s="7"/>
       <c r="F64" s="7"/>
@@ -2619,10 +2637,10 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="B65" s="7" t="s">
         <v>220</v>
-      </c>
-      <c r="B65" s="7" t="s">
-        <v>214</v>
       </c>
       <c r="C65" s="8" t="s">
         <v>221</v>
@@ -2640,7 +2658,7 @@
         <v>223</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C66" s="8" t="s">
         <v>224</v>
@@ -2658,7 +2676,7 @@
         <v>226</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C67" s="8" t="s">
         <v>227</v>
@@ -2676,7 +2694,7 @@
         <v>229</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C68" s="8" t="s">
         <v>230</v>
@@ -2694,7 +2712,7 @@
         <v>232</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C69" s="8" t="s">
         <v>233</v>
@@ -2712,7 +2730,7 @@
         <v>235</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C70" s="8" t="s">
         <v>236</v>
@@ -2730,7 +2748,7 @@
         <v>238</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C71" s="8" t="s">
         <v>239</v>
@@ -2748,13 +2766,13 @@
         <v>241</v>
       </c>
       <c r="B72" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="C72" s="8" t="s">
         <v>242</v>
       </c>
-      <c r="C72" s="8" t="s">
+      <c r="D72" s="8" t="s">
         <v>243</v>
-      </c>
-      <c r="D72" s="8" t="s">
-        <v>244</v>
       </c>
       <c r="E72" s="7"/>
       <c r="F72" s="7"/>
@@ -2763,16 +2781,16 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="B73" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="C73" s="8" t="s">
         <v>245</v>
       </c>
-      <c r="B73" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="C73" s="8" t="s">
+      <c r="D73" s="8" t="s">
         <v>246</v>
-      </c>
-      <c r="D73" s="8" t="s">
-        <v>247</v>
       </c>
       <c r="E73" s="7"/>
       <c r="F73" s="7"/>
@@ -2781,10 +2799,10 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="B74" s="7" t="s">
         <v>248</v>
-      </c>
-      <c r="B74" s="7" t="s">
-        <v>242</v>
       </c>
       <c r="C74" s="8" t="s">
         <v>249</v>
@@ -2802,13 +2820,13 @@
         <v>251</v>
       </c>
       <c r="B75" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="C75" s="8" t="s">
         <v>252</v>
       </c>
-      <c r="C75" s="8" t="s">
+      <c r="D75" s="8" t="s">
         <v>253</v>
-      </c>
-      <c r="D75" s="8" t="s">
-        <v>254</v>
       </c>
       <c r="E75" s="7"/>
       <c r="F75" s="7"/>
@@ -2817,16 +2835,16 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="B76" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="C76" s="8" t="s">
         <v>255</v>
       </c>
-      <c r="B76" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="C76" s="8" t="s">
+      <c r="D76" s="8" t="s">
         <v>256</v>
-      </c>
-      <c r="D76" s="8" t="s">
-        <v>257</v>
       </c>
       <c r="E76" s="7"/>
       <c r="F76" s="7"/>
@@ -2835,10 +2853,10 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="B77" s="7" t="s">
         <v>258</v>
-      </c>
-      <c r="B77" s="7" t="s">
-        <v>252</v>
       </c>
       <c r="C77" s="8" t="s">
         <v>259</v>
@@ -2856,7 +2874,7 @@
         <v>261</v>
       </c>
       <c r="B78" s="7" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="C78" s="8" t="s">
         <v>262</v>
@@ -2874,7 +2892,7 @@
         <v>264</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="C79" s="8" t="s">
         <v>265</v>
@@ -2892,13 +2910,13 @@
         <v>267</v>
       </c>
       <c r="B80" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="C80" s="8" t="s">
         <v>268</v>
       </c>
-      <c r="C80" s="8" t="s">
+      <c r="D80" s="8" t="s">
         <v>269</v>
-      </c>
-      <c r="D80" s="8" t="s">
-        <v>270</v>
       </c>
       <c r="E80" s="7"/>
       <c r="F80" s="7"/>
@@ -2907,16 +2925,16 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="B81" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="C81" s="8" t="s">
         <v>271</v>
       </c>
-      <c r="B81" s="7" t="s">
-        <v>268</v>
-      </c>
-      <c r="C81" s="8" t="s">
+      <c r="D81" s="8" t="s">
         <v>272</v>
-      </c>
-      <c r="D81" s="8" t="s">
-        <v>273</v>
       </c>
       <c r="E81" s="7"/>
       <c r="F81" s="7"/>
@@ -2925,16 +2943,16 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="B82" s="7" t="s">
         <v>274</v>
       </c>
-      <c r="B82" s="7" t="s">
+      <c r="C82" s="8" t="s">
         <v>275</v>
       </c>
-      <c r="C82" s="8" t="s">
+      <c r="D82" s="8" t="s">
         <v>276</v>
-      </c>
-      <c r="D82" s="8" t="s">
-        <v>277</v>
       </c>
       <c r="E82" s="7"/>
       <c r="F82" s="7"/>
@@ -2943,16 +2961,16 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="B83" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="C83" s="8" t="s">
         <v>278</v>
       </c>
-      <c r="B83" s="7" t="s">
-        <v>275</v>
-      </c>
-      <c r="C83" s="8" t="s">
+      <c r="D83" s="8" t="s">
         <v>279</v>
-      </c>
-      <c r="D83" s="8" t="s">
-        <v>280</v>
       </c>
       <c r="E83" s="7"/>
       <c r="F83" s="7"/>
@@ -2961,16 +2979,16 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="B84" s="7" t="s">
         <v>281</v>
-      </c>
-      <c r="B84" s="7" t="s">
-        <v>275</v>
       </c>
       <c r="C84" s="8" t="s">
         <v>282</v>
       </c>
       <c r="D84" s="8" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="E84" s="7"/>
       <c r="F84" s="7"/>
@@ -2979,16 +2997,16 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="7" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B85" s="7" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="C85" s="8" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D85" s="8" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="E85" s="7"/>
       <c r="F85" s="7"/>
@@ -2997,26 +3015,62 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="7" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B86" s="7" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="C86" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="D86" s="8" t="s">
         <v>286</v>
-      </c>
-      <c r="D86" s="8" t="s">
-        <v>280</v>
       </c>
       <c r="E86" s="7"/>
       <c r="F86" s="7"/>
       <c r="G86" s="7"/>
       <c r="H86" s="8"/>
     </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="B87" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="C87" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="D87" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="E87" s="7"/>
+      <c r="F87" s="7"/>
+      <c r="G87" s="7"/>
+      <c r="H87" s="8"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="B88" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>292</v>
+      </c>
+      <c r="D88" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="E88" s="7"/>
+      <c r="F88" s="7"/>
+      <c r="G88" s="7"/>
+      <c r="H88" s="8"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H86"/>
+  <autoFilter ref="A1:H88"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E86" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E88" type="list">
       <formula1>"Pass,Fail,Blocked,N/A"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Add generate_firmware_report (firmware compliance) + docs - v1.13.0
</commit_message>
<xml_diff>
--- a/TEST_RESULTS_TRACKER.xlsx
+++ b/TEST_RESULTS_TRACKER.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Test Results" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Results'!$A$1:$H$88</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Results'!$A$1:$H$89</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="296">
   <si>
     <t xml:space="preserve">HPE Networking Assistant — Test Results Summary</t>
   </si>
@@ -143,7 +143,7 @@
     <t xml:space="preserve">Run pytest -q</t>
   </si>
   <si>
-    <t xml:space="preserve">87 passed</t>
+    <t xml:space="preserve">90 passed</t>
   </si>
   <si>
     <t xml:space="preserve">A3</t>
@@ -482,6 +482,15 @@
     <t xml:space="preserve">PDF produced from Markdown</t>
   </si>
   <si>
+    <t xml:space="preserve">RPT-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">generate_firmware_report</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-model target version + devices behind it</t>
+  </si>
+  <si>
     <t xml:space="preserve">CT-1</t>
   </si>
   <si>
@@ -902,7 +911,7 @@
     <t xml:space="preserve">SC-5</t>
   </si>
   <si>
-    <t xml:space="preserve">Automated suite 87 passed</t>
+    <t xml:space="preserve">Automated suite 90 passed</t>
   </si>
 </sst>
 </file>
@@ -1389,8 +1398,8 @@
         <v>7</v>
       </c>
       <c r="B9" s="3" t="n">
-        <f aca="false">COUNTA('Test Results'!A2:A88)</f>
-        <v>87</v>
+        <f aca="false">COUNTA('Test Results'!A2:A89)</f>
+        <v>88</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1398,7 +1407,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E88,"Pass")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E89,"Pass")</f>
         <v>0</v>
       </c>
     </row>
@@ -1407,7 +1416,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E88,"Fail")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E89,"Fail")</f>
         <v>0</v>
       </c>
     </row>
@@ -1416,7 +1425,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E88,"Blocked")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E89,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
@@ -1425,7 +1434,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E88,"N/A")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E89,"N/A")</f>
         <v>0</v>
       </c>
     </row>
@@ -1435,7 +1444,7 @@
       </c>
       <c r="B14" s="3" t="n">
         <f aca="false">B9-(B10+B11+B12+B13)</f>
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1463,7 +1472,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H89"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -2262,13 +2271,13 @@
         <v>152</v>
       </c>
       <c r="B44" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="C44" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="C44" s="8" t="s">
+      <c r="D44" s="8" t="s">
         <v>154</v>
-      </c>
-      <c r="D44" s="8" t="s">
-        <v>155</v>
       </c>
       <c r="E44" s="7"/>
       <c r="F44" s="7"/>
@@ -2277,10 +2286,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B45" s="7" t="s">
         <v>156</v>
-      </c>
-      <c r="B45" s="7" t="s">
-        <v>153</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>157</v>
@@ -2298,7 +2307,7 @@
         <v>159</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="C46" s="8" t="s">
         <v>160</v>
@@ -2316,7 +2325,7 @@
         <v>162</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>163</v>
@@ -2334,13 +2343,13 @@
         <v>165</v>
       </c>
       <c r="B48" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="C48" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="C48" s="8" t="s">
+      <c r="D48" s="8" t="s">
         <v>167</v>
-      </c>
-      <c r="D48" s="8" t="s">
-        <v>168</v>
       </c>
       <c r="E48" s="7"/>
       <c r="F48" s="7"/>
@@ -2349,10 +2358,10 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="B49" s="7" t="s">
         <v>169</v>
-      </c>
-      <c r="B49" s="7" t="s">
-        <v>166</v>
       </c>
       <c r="C49" s="8" t="s">
         <v>170</v>
@@ -2370,7 +2379,7 @@
         <v>172</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>173</v>
@@ -2388,7 +2397,7 @@
         <v>175</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C51" s="8" t="s">
         <v>176</v>
@@ -2401,12 +2410,12 @@
       <c r="G51" s="7"/>
       <c r="H51" s="8"/>
     </row>
-    <row r="52" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
         <v>178</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>179</v>
@@ -2419,18 +2428,18 @@
       <c r="G52" s="7"/>
       <c r="H52" s="8"/>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
         <v>181</v>
       </c>
       <c r="B53" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="C53" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="C53" s="8" t="s">
+      <c r="D53" s="8" t="s">
         <v>183</v>
-      </c>
-      <c r="D53" s="8" t="s">
-        <v>184</v>
       </c>
       <c r="E53" s="7"/>
       <c r="F53" s="7"/>
@@ -2439,10 +2448,10 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="B54" s="7" t="s">
         <v>185</v>
-      </c>
-      <c r="B54" s="7" t="s">
-        <v>182</v>
       </c>
       <c r="C54" s="8" t="s">
         <v>186</v>
@@ -2460,7 +2469,7 @@
         <v>188</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C55" s="8" t="s">
         <v>189</v>
@@ -2478,7 +2487,7 @@
         <v>191</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C56" s="8" t="s">
         <v>192</v>
@@ -2496,25 +2505,25 @@
         <v>194</v>
       </c>
       <c r="B57" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C57" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="C57" s="8" t="s">
+      <c r="D57" s="8" t="s">
         <v>196</v>
-      </c>
-      <c r="D57" s="8" t="s">
-        <v>197</v>
       </c>
       <c r="E57" s="7"/>
       <c r="F57" s="7"/>
       <c r="G57" s="7"/>
       <c r="H57" s="8"/>
     </row>
-    <row r="58" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="B58" s="7" t="s">
         <v>198</v>
-      </c>
-      <c r="B58" s="7" t="s">
-        <v>195</v>
       </c>
       <c r="C58" s="8" t="s">
         <v>199</v>
@@ -2527,12 +2536,12 @@
       <c r="G58" s="7"/>
       <c r="H58" s="8"/>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
         <v>201</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C59" s="8" t="s">
         <v>202</v>
@@ -2550,7 +2559,7 @@
         <v>204</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C60" s="8" t="s">
         <v>205</v>
@@ -2563,12 +2572,12 @@
       <c r="G60" s="7"/>
       <c r="H60" s="8"/>
     </row>
-    <row r="61" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
         <v>207</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C61" s="8" t="s">
         <v>208</v>
@@ -2581,12 +2590,12 @@
       <c r="G61" s="7"/>
       <c r="H61" s="8"/>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
         <v>210</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C62" s="8" t="s">
         <v>211</v>
@@ -2599,12 +2608,12 @@
       <c r="G62" s="7"/>
       <c r="H62" s="8"/>
     </row>
-    <row r="63" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
         <v>213</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C63" s="8" t="s">
         <v>214</v>
@@ -2617,12 +2626,12 @@
       <c r="G63" s="7"/>
       <c r="H63" s="8"/>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
         <v>216</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C64" s="8" t="s">
         <v>217</v>
@@ -2640,13 +2649,13 @@
         <v>219</v>
       </c>
       <c r="B65" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="C65" s="8" t="s">
         <v>220</v>
       </c>
-      <c r="C65" s="8" t="s">
+      <c r="D65" s="8" t="s">
         <v>221</v>
-      </c>
-      <c r="D65" s="8" t="s">
-        <v>222</v>
       </c>
       <c r="E65" s="7"/>
       <c r="F65" s="7"/>
@@ -2655,10 +2664,10 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="B66" s="7" t="s">
         <v>223</v>
-      </c>
-      <c r="B66" s="7" t="s">
-        <v>220</v>
       </c>
       <c r="C66" s="8" t="s">
         <v>224</v>
@@ -2676,7 +2685,7 @@
         <v>226</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C67" s="8" t="s">
         <v>227</v>
@@ -2694,7 +2703,7 @@
         <v>229</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C68" s="8" t="s">
         <v>230</v>
@@ -2712,7 +2721,7 @@
         <v>232</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C69" s="8" t="s">
         <v>233</v>
@@ -2730,7 +2739,7 @@
         <v>235</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C70" s="8" t="s">
         <v>236</v>
@@ -2748,7 +2757,7 @@
         <v>238</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C71" s="8" t="s">
         <v>239</v>
@@ -2766,7 +2775,7 @@
         <v>241</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C72" s="8" t="s">
         <v>242</v>
@@ -2784,7 +2793,7 @@
         <v>244</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C73" s="8" t="s">
         <v>245</v>
@@ -2802,13 +2811,13 @@
         <v>247</v>
       </c>
       <c r="B74" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="C74" s="8" t="s">
         <v>248</v>
       </c>
-      <c r="C74" s="8" t="s">
+      <c r="D74" s="8" t="s">
         <v>249</v>
-      </c>
-      <c r="D74" s="8" t="s">
-        <v>250</v>
       </c>
       <c r="E74" s="7"/>
       <c r="F74" s="7"/>
@@ -2817,10 +2826,10 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="B75" s="7" t="s">
         <v>251</v>
-      </c>
-      <c r="B75" s="7" t="s">
-        <v>248</v>
       </c>
       <c r="C75" s="8" t="s">
         <v>252</v>
@@ -2838,7 +2847,7 @@
         <v>254</v>
       </c>
       <c r="B76" s="7" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="C76" s="8" t="s">
         <v>255</v>
@@ -2856,13 +2865,13 @@
         <v>257</v>
       </c>
       <c r="B77" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="C77" s="8" t="s">
         <v>258</v>
       </c>
-      <c r="C77" s="8" t="s">
+      <c r="D77" s="8" t="s">
         <v>259</v>
-      </c>
-      <c r="D77" s="8" t="s">
-        <v>260</v>
       </c>
       <c r="E77" s="7"/>
       <c r="F77" s="7"/>
@@ -2871,10 +2880,10 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="B78" s="7" t="s">
         <v>261</v>
-      </c>
-      <c r="B78" s="7" t="s">
-        <v>258</v>
       </c>
       <c r="C78" s="8" t="s">
         <v>262</v>
@@ -2892,7 +2901,7 @@
         <v>264</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="C79" s="8" t="s">
         <v>265</v>
@@ -2910,7 +2919,7 @@
         <v>267</v>
       </c>
       <c r="B80" s="7" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="C80" s="8" t="s">
         <v>268</v>
@@ -2928,7 +2937,7 @@
         <v>270</v>
       </c>
       <c r="B81" s="7" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="C81" s="8" t="s">
         <v>271</v>
@@ -2946,13 +2955,13 @@
         <v>273</v>
       </c>
       <c r="B82" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="C82" s="8" t="s">
         <v>274</v>
       </c>
-      <c r="C82" s="8" t="s">
+      <c r="D82" s="8" t="s">
         <v>275</v>
-      </c>
-      <c r="D82" s="8" t="s">
-        <v>276</v>
       </c>
       <c r="E82" s="7"/>
       <c r="F82" s="7"/>
@@ -2961,10 +2970,10 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="B83" s="7" t="s">
         <v>277</v>
-      </c>
-      <c r="B83" s="7" t="s">
-        <v>274</v>
       </c>
       <c r="C83" s="8" t="s">
         <v>278</v>
@@ -2982,13 +2991,13 @@
         <v>280</v>
       </c>
       <c r="B84" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C84" s="8" t="s">
         <v>281</v>
       </c>
-      <c r="C84" s="8" t="s">
+      <c r="D84" s="8" t="s">
         <v>282</v>
-      </c>
-      <c r="D84" s="8" t="s">
-        <v>283</v>
       </c>
       <c r="E84" s="7"/>
       <c r="F84" s="7"/>
@@ -2997,10 +3006,10 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="B85" s="7" t="s">
         <v>284</v>
-      </c>
-      <c r="B85" s="7" t="s">
-        <v>281</v>
       </c>
       <c r="C85" s="8" t="s">
         <v>285</v>
@@ -3018,13 +3027,13 @@
         <v>287</v>
       </c>
       <c r="B86" s="7" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="C86" s="8" t="s">
         <v>288</v>
       </c>
       <c r="D86" s="8" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E86" s="7"/>
       <c r="F86" s="7"/>
@@ -3033,16 +3042,16 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="B87" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="C87" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="D87" s="8" t="s">
         <v>289</v>
-      </c>
-      <c r="B87" s="7" t="s">
-        <v>281</v>
-      </c>
-      <c r="C87" s="8" t="s">
-        <v>290</v>
-      </c>
-      <c r="D87" s="8" t="s">
-        <v>286</v>
       </c>
       <c r="E87" s="7"/>
       <c r="F87" s="7"/>
@@ -3051,26 +3060,44 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="7" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B88" s="7" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="C88" s="8" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D88" s="8" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E88" s="7"/>
       <c r="F88" s="7"/>
       <c r="G88" s="7"/>
       <c r="H88" s="8"/>
     </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="B89" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="C89" s="8" t="s">
+        <v>295</v>
+      </c>
+      <c r="D89" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="E89" s="7"/>
+      <c r="F89" s="7"/>
+      <c r="G89" s="7"/>
+      <c r="H89" s="8"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H88"/>
+  <autoFilter ref="A1:H89"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E88" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E89" type="list">
       <formula1>"Pass,Fail,Blocked,N/A"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Add generate_topology (per-site Mermaid network topology) + docs - v1.14.0
</commit_message>
<xml_diff>
--- a/TEST_RESULTS_TRACKER.xlsx
+++ b/TEST_RESULTS_TRACKER.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Test Results" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Results'!$A$1:$H$89</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Results'!$A$1:$H$90</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="299">
   <si>
     <t xml:space="preserve">HPE Networking Assistant — Test Results Summary</t>
   </si>
@@ -143,7 +143,7 @@
     <t xml:space="preserve">Run pytest -q</t>
   </si>
   <si>
-    <t xml:space="preserve">90 passed</t>
+    <t xml:space="preserve">95 passed</t>
   </si>
   <si>
     <t xml:space="preserve">A3</t>
@@ -491,6 +491,15 @@
     <t xml:space="preserve">Per-model target version + devices behind it</t>
   </si>
   <si>
+    <t xml:space="preserve">RPT-7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">generate_topology</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-site Mermaid topology (gw/switch/AP via LLDP) + counts</t>
+  </si>
+  <si>
     <t xml:space="preserve">CT-1</t>
   </si>
   <si>
@@ -911,7 +920,7 @@
     <t xml:space="preserve">SC-5</t>
   </si>
   <si>
-    <t xml:space="preserve">Automated suite 90 passed</t>
+    <t xml:space="preserve">Automated suite 95 passed</t>
   </si>
 </sst>
 </file>
@@ -1398,8 +1407,8 @@
         <v>7</v>
       </c>
       <c r="B9" s="3" t="n">
-        <f aca="false">COUNTA('Test Results'!A2:A89)</f>
-        <v>88</v>
+        <f aca="false">COUNTA('Test Results'!A2:A90)</f>
+        <v>89</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1407,7 +1416,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E89,"Pass")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E90,"Pass")</f>
         <v>0</v>
       </c>
     </row>
@@ -1416,7 +1425,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E89,"Fail")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E90,"Fail")</f>
         <v>0</v>
       </c>
     </row>
@@ -1425,7 +1434,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E89,"Blocked")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E90,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
@@ -1434,7 +1443,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="3" t="n">
-        <f aca="false">COUNTIF('Test Results'!E2:E89,"N/A")</f>
+        <f aca="false">COUNTIF('Test Results'!E2:E90,"N/A")</f>
         <v>0</v>
       </c>
     </row>
@@ -1444,7 +1453,7 @@
       </c>
       <c r="B14" s="3" t="n">
         <f aca="false">B9-(B10+B11+B12+B13)</f>
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1472,7 +1481,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H89"/>
+  <dimension ref="A1:H90"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -2284,18 +2293,18 @@
       <c r="G44" s="7"/>
       <c r="H44" s="8"/>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
         <v>155</v>
       </c>
       <c r="B45" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="C45" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="C45" s="8" t="s">
+      <c r="D45" s="8" t="s">
         <v>157</v>
-      </c>
-      <c r="D45" s="8" t="s">
-        <v>158</v>
       </c>
       <c r="E45" s="7"/>
       <c r="F45" s="7"/>
@@ -2304,10 +2313,10 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B46" s="7" t="s">
         <v>159</v>
-      </c>
-      <c r="B46" s="7" t="s">
-        <v>156</v>
       </c>
       <c r="C46" s="8" t="s">
         <v>160</v>
@@ -2325,7 +2334,7 @@
         <v>162</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>163</v>
@@ -2343,7 +2352,7 @@
         <v>165</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C48" s="8" t="s">
         <v>166</v>
@@ -2361,13 +2370,13 @@
         <v>168</v>
       </c>
       <c r="B49" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="C49" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="C49" s="8" t="s">
+      <c r="D49" s="8" t="s">
         <v>170</v>
-      </c>
-      <c r="D49" s="8" t="s">
-        <v>171</v>
       </c>
       <c r="E49" s="7"/>
       <c r="F49" s="7"/>
@@ -2376,10 +2385,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="B50" s="7" t="s">
         <v>172</v>
-      </c>
-      <c r="B50" s="7" t="s">
-        <v>169</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>173</v>
@@ -2397,7 +2406,7 @@
         <v>175</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C51" s="8" t="s">
         <v>176</v>
@@ -2415,7 +2424,7 @@
         <v>178</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>179</v>
@@ -2428,12 +2437,12 @@
       <c r="G52" s="7"/>
       <c r="H52" s="8"/>
     </row>
-    <row r="53" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
         <v>181</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C53" s="8" t="s">
         <v>182</v>
@@ -2446,18 +2455,18 @@
       <c r="G53" s="7"/>
       <c r="H53" s="8"/>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
         <v>184</v>
       </c>
       <c r="B54" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="C54" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="C54" s="8" t="s">
+      <c r="D54" s="8" t="s">
         <v>186</v>
-      </c>
-      <c r="D54" s="8" t="s">
-        <v>187</v>
       </c>
       <c r="E54" s="7"/>
       <c r="F54" s="7"/>
@@ -2466,10 +2475,10 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="B55" s="7" t="s">
         <v>188</v>
-      </c>
-      <c r="B55" s="7" t="s">
-        <v>185</v>
       </c>
       <c r="C55" s="8" t="s">
         <v>189</v>
@@ -2487,7 +2496,7 @@
         <v>191</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C56" s="8" t="s">
         <v>192</v>
@@ -2505,7 +2514,7 @@
         <v>194</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C57" s="8" t="s">
         <v>195</v>
@@ -2523,25 +2532,25 @@
         <v>197</v>
       </c>
       <c r="B58" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="C58" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="C58" s="8" t="s">
+      <c r="D58" s="8" t="s">
         <v>199</v>
-      </c>
-      <c r="D58" s="8" t="s">
-        <v>200</v>
       </c>
       <c r="E58" s="7"/>
       <c r="F58" s="7"/>
       <c r="G58" s="7"/>
       <c r="H58" s="8"/>
     </row>
-    <row r="59" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="B59" s="7" t="s">
         <v>201</v>
-      </c>
-      <c r="B59" s="7" t="s">
-        <v>198</v>
       </c>
       <c r="C59" s="8" t="s">
         <v>202</v>
@@ -2554,12 +2563,12 @@
       <c r="G59" s="7"/>
       <c r="H59" s="8"/>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
         <v>204</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C60" s="8" t="s">
         <v>205</v>
@@ -2577,7 +2586,7 @@
         <v>207</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C61" s="8" t="s">
         <v>208</v>
@@ -2590,12 +2599,12 @@
       <c r="G61" s="7"/>
       <c r="H61" s="8"/>
     </row>
-    <row r="62" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
         <v>210</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C62" s="8" t="s">
         <v>211</v>
@@ -2608,12 +2617,12 @@
       <c r="G62" s="7"/>
       <c r="H62" s="8"/>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
         <v>213</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C63" s="8" t="s">
         <v>214</v>
@@ -2626,12 +2635,12 @@
       <c r="G63" s="7"/>
       <c r="H63" s="8"/>
     </row>
-    <row r="64" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
         <v>216</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C64" s="8" t="s">
         <v>217</v>
@@ -2644,12 +2653,12 @@
       <c r="G64" s="7"/>
       <c r="H64" s="8"/>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
         <v>219</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C65" s="8" t="s">
         <v>220</v>
@@ -2667,13 +2676,13 @@
         <v>222</v>
       </c>
       <c r="B66" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="C66" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="C66" s="8" t="s">
+      <c r="D66" s="8" t="s">
         <v>224</v>
-      </c>
-      <c r="D66" s="8" t="s">
-        <v>225</v>
       </c>
       <c r="E66" s="7"/>
       <c r="F66" s="7"/>
@@ -2682,10 +2691,10 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="B67" s="7" t="s">
         <v>226</v>
-      </c>
-      <c r="B67" s="7" t="s">
-        <v>223</v>
       </c>
       <c r="C67" s="8" t="s">
         <v>227</v>
@@ -2703,7 +2712,7 @@
         <v>229</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C68" s="8" t="s">
         <v>230</v>
@@ -2721,7 +2730,7 @@
         <v>232</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C69" s="8" t="s">
         <v>233</v>
@@ -2739,7 +2748,7 @@
         <v>235</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C70" s="8" t="s">
         <v>236</v>
@@ -2757,7 +2766,7 @@
         <v>238</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C71" s="8" t="s">
         <v>239</v>
@@ -2775,7 +2784,7 @@
         <v>241</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C72" s="8" t="s">
         <v>242</v>
@@ -2793,7 +2802,7 @@
         <v>244</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C73" s="8" t="s">
         <v>245</v>
@@ -2811,7 +2820,7 @@
         <v>247</v>
       </c>
       <c r="B74" s="7" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C74" s="8" t="s">
         <v>248</v>
@@ -2829,13 +2838,13 @@
         <v>250</v>
       </c>
       <c r="B75" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="C75" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="C75" s="8" t="s">
+      <c r="D75" s="8" t="s">
         <v>252</v>
-      </c>
-      <c r="D75" s="8" t="s">
-        <v>253</v>
       </c>
       <c r="E75" s="7"/>
       <c r="F75" s="7"/>
@@ -2844,10 +2853,10 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="B76" s="7" t="s">
         <v>254</v>
-      </c>
-      <c r="B76" s="7" t="s">
-        <v>251</v>
       </c>
       <c r="C76" s="8" t="s">
         <v>255</v>
@@ -2865,7 +2874,7 @@
         <v>257</v>
       </c>
       <c r="B77" s="7" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="C77" s="8" t="s">
         <v>258</v>
@@ -2883,13 +2892,13 @@
         <v>260</v>
       </c>
       <c r="B78" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="C78" s="8" t="s">
         <v>261</v>
       </c>
-      <c r="C78" s="8" t="s">
+      <c r="D78" s="8" t="s">
         <v>262</v>
-      </c>
-      <c r="D78" s="8" t="s">
-        <v>263</v>
       </c>
       <c r="E78" s="7"/>
       <c r="F78" s="7"/>
@@ -2898,10 +2907,10 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="B79" s="7" t="s">
         <v>264</v>
-      </c>
-      <c r="B79" s="7" t="s">
-        <v>261</v>
       </c>
       <c r="C79" s="8" t="s">
         <v>265</v>
@@ -2919,7 +2928,7 @@
         <v>267</v>
       </c>
       <c r="B80" s="7" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C80" s="8" t="s">
         <v>268</v>
@@ -2937,7 +2946,7 @@
         <v>270</v>
       </c>
       <c r="B81" s="7" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C81" s="8" t="s">
         <v>271</v>
@@ -2955,7 +2964,7 @@
         <v>273</v>
       </c>
       <c r="B82" s="7" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C82" s="8" t="s">
         <v>274</v>
@@ -2973,13 +2982,13 @@
         <v>276</v>
       </c>
       <c r="B83" s="7" t="s">
+        <v>264</v>
+      </c>
+      <c r="C83" s="8" t="s">
         <v>277</v>
       </c>
-      <c r="C83" s="8" t="s">
+      <c r="D83" s="8" t="s">
         <v>278</v>
-      </c>
-      <c r="D83" s="8" t="s">
-        <v>279</v>
       </c>
       <c r="E83" s="7"/>
       <c r="F83" s="7"/>
@@ -2988,10 +2997,10 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="B84" s="7" t="s">
         <v>280</v>
-      </c>
-      <c r="B84" s="7" t="s">
-        <v>277</v>
       </c>
       <c r="C84" s="8" t="s">
         <v>281</v>
@@ -3009,13 +3018,13 @@
         <v>283</v>
       </c>
       <c r="B85" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="C85" s="8" t="s">
         <v>284</v>
       </c>
-      <c r="C85" s="8" t="s">
+      <c r="D85" s="8" t="s">
         <v>285</v>
-      </c>
-      <c r="D85" s="8" t="s">
-        <v>286</v>
       </c>
       <c r="E85" s="7"/>
       <c r="F85" s="7"/>
@@ -3024,10 +3033,10 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="B86" s="7" t="s">
         <v>287</v>
-      </c>
-      <c r="B86" s="7" t="s">
-        <v>284</v>
       </c>
       <c r="C86" s="8" t="s">
         <v>288</v>
@@ -3045,13 +3054,13 @@
         <v>290</v>
       </c>
       <c r="B87" s="7" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="C87" s="8" t="s">
         <v>291</v>
       </c>
       <c r="D87" s="8" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E87" s="7"/>
       <c r="F87" s="7"/>
@@ -3060,16 +3069,16 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="B88" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="D88" s="8" t="s">
         <v>292</v>
-      </c>
-      <c r="B88" s="7" t="s">
-        <v>284</v>
-      </c>
-      <c r="C88" s="8" t="s">
-        <v>293</v>
-      </c>
-      <c r="D88" s="8" t="s">
-        <v>289</v>
       </c>
       <c r="E88" s="7"/>
       <c r="F88" s="7"/>
@@ -3078,26 +3087,44 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="7" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B89" s="7" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="C89" s="8" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D89" s="8" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E89" s="7"/>
       <c r="F89" s="7"/>
       <c r="G89" s="7"/>
       <c r="H89" s="8"/>
     </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="B90" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="D90" s="8" t="s">
+        <v>292</v>
+      </c>
+      <c r="E90" s="7"/>
+      <c r="F90" s="7"/>
+      <c r="G90" s="7"/>
+      <c r="H90" s="8"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H89"/>
+  <autoFilter ref="A1:H90"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E89" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E90" type="list">
       <formula1>"Pass,Fail,Blocked,N/A"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>